<commit_message>
corpus: regenerate every zone-carrying input as v21 (Type words, not sentinels)
The seven files that carry SSR overlays — vp040 (three 'ssr elastic'), vp102a and the
five vp102t_* drawdown snapshots ('ssr reduce') — are rebuilt through their own builders,
so the overlays are now written as Type words instead of negative Mat IDs. The zones are
semantically identical, and the loader reads either forever.

The vp102t rebuild re-solves the 1500 h transient that produces its u='seep' sidecars.
All eleven sidecars and meshes come back BYTE-IDENTICAL, so only the .xlsx changed and
nothing physical moved. verify_rebuild is green on problems + rs2 (181/181).

Also syncs the packaged copy of the modeling skill (template_sync).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/vp040.xlsx
+++ b/docs/verification/files/rocscience/vp040.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8D9778-BA48-644C-980F-473DF9F954B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EEB53F3-5E86-5B42-A7B6-55B20E1E8D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="34200" windowHeight="19900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="310">
   <si>
     <t>time</t>
   </si>
@@ -971,7 +971,25 @@
     <t>corps</t>
   </si>
   <si>
-    <t>Mat ID = -1 --&gt; SSR reduce, Mat ID = -2 --&gt; SSR hold, Mat ID = -3 --&gt; SSR elastic</t>
+    <t>Size:</t>
+  </si>
+  <si>
+    <t>Direction:</t>
+  </si>
+  <si>
+    <t>material</t>
+  </si>
+  <si>
+    <t>Type: material zone (default), an SSR analysis overlay, or a mesh refinement region.   Size: optional target mesh element size inside the polygon (blank = global size).</t>
+  </si>
+  <si>
+    <t>Side BC:</t>
+  </si>
+  <si>
+    <t>rollers</t>
+  </si>
+  <si>
+    <t>Size: optional target mesh element size inside this line's material zone (blank = global size).</t>
   </si>
 </sst>
 </file>
@@ -1479,18 +1497,11 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="35">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1511,7 +1522,119 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1686,7 +1809,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$A$8:$A$27</c:f>
+              <c:f>profile!$A$9:$A$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1695,7 +1818,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$B$8:$B$27</c:f>
+              <c:f>profile!$B$9:$B$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1749,7 +1872,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$D$8:$D$27</c:f>
+              <c:f>profile!$D$9:$D$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1758,7 +1881,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$E$8:$E$27</c:f>
+              <c:f>profile!$E$9:$E$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1812,7 +1935,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$G$8:$G$27</c:f>
+              <c:f>profile!$G$9:$G$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1821,7 +1944,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$H$8:$H$27</c:f>
+              <c:f>profile!$H$9:$H$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1875,7 +1998,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$J$8:$J$27</c:f>
+              <c:f>profile!$J$9:$J$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1884,7 +2007,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$K$8:$K$27</c:f>
+              <c:f>profile!$K$9:$K$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1938,7 +2061,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$M$8:$M$27</c:f>
+              <c:f>profile!$M$9:$M$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1947,7 +2070,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$N$8:$N$27</c:f>
+              <c:f>profile!$N$9:$N$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2001,7 +2124,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$P$8:$P$27</c:f>
+              <c:f>profile!$P$9:$P$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2010,7 +2133,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$Q$8:$Q$27</c:f>
+              <c:f>profile!$Q$9:$Q$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2070,7 +2193,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$S$8:$S$27</c:f>
+              <c:f>profile!$S$9:$S$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2079,7 +2202,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$T$8:$T$27</c:f>
+              <c:f>profile!$T$9:$T$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2139,7 +2262,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$V$8:$V$27</c:f>
+              <c:f>profile!$V$9:$V$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2148,7 +2271,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$W$8:$W$27</c:f>
+              <c:f>profile!$W$9:$W$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2208,7 +2331,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$Y$8:$Y$27</c:f>
+              <c:f>profile!$Y$9:$Y$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2217,7 +2340,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$Z$8:$Z$27</c:f>
+              <c:f>profile!$Z$9:$Z$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2277,7 +2400,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AB$8:$AB$27</c:f>
+              <c:f>profile!$AB$9:$AB$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2286,7 +2409,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AC$8:$AC$27</c:f>
+              <c:f>profile!$AC$9:$AC$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2346,7 +2469,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AE$8:$AE$27</c:f>
+              <c:f>profile!$AE$9:$AE$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2355,7 +2478,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AF$8:$AF$27</c:f>
+              <c:f>profile!$AF$9:$AF$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2415,7 +2538,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AH$8:$AH$27</c:f>
+              <c:f>profile!$AH$9:$AH$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2424,7 +2547,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AI$8:$AI$27</c:f>
+              <c:f>profile!$AI$9:$AI$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2484,7 +2607,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AK$8:$AK$27</c:f>
+              <c:f>profile!$AK$9:$AK$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2493,7 +2616,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AL$8:$AL$27</c:f>
+              <c:f>profile!$AL$9:$AL$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2556,7 +2679,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AN$8:$AN$27</c:f>
+              <c:f>profile!$AN$9:$AN$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2565,7 +2688,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AO$8:$AO$27</c:f>
+              <c:f>profile!$AO$9:$AO$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2628,7 +2751,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AQ$8:$AQ$27</c:f>
+              <c:f>profile!$AQ$9:$AQ$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2637,7 +2760,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AR$8:$AR$27</c:f>
+              <c:f>profile!$AR$9:$AR$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2879,7 +3002,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$B$4:$B$13</c:f>
+              <c:f>dloads!$B$5:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2888,7 +3011,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$C$4:$C$13</c:f>
+              <c:f>dloads!$C$5:$C$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2951,7 +3074,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$F$4:$F$13</c:f>
+              <c:f>dloads!$F$5:$F$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2960,7 +3083,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$G$4:$G$13</c:f>
+              <c:f>dloads!$G$5:$G$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3023,7 +3146,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$J$4:$J$13</c:f>
+              <c:f>dloads!$J$5:$J$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3032,7 +3155,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$K$4:$K$13</c:f>
+              <c:f>dloads!$K$5:$K$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3095,7 +3218,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$N$4:$N$13</c:f>
+              <c:f>dloads!$N$5:$N$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3104,7 +3227,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$O$4:$O$13</c:f>
+              <c:f>dloads!$O$5:$O$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3167,7 +3290,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$R$4:$R$22</c:f>
+              <c:f>dloads!$R$5:$R$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3176,7 +3299,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$S$4:$S$22</c:f>
+              <c:f>dloads!$S$5:$S$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3239,7 +3362,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$V$4:$V$22</c:f>
+              <c:f>dloads!$V$5:$V$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3248,7 +3371,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$W$4:$W$22</c:f>
+              <c:f>dloads!$W$5:$W$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3496,7 +3619,7 @@
           </c:dPt>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$B$4:$B$22</c:f>
+              <c:f>'dloads (2)'!$B$5:$B$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3505,7 +3628,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$C$4:$C$22</c:f>
+              <c:f>'dloads (2)'!$C$5:$C$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3565,7 +3688,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$F$4:$F$22</c:f>
+              <c:f>'dloads (2)'!$F$5:$F$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3574,7 +3697,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$G$4:$G$22</c:f>
+              <c:f>'dloads (2)'!$G$5:$G$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3628,7 +3751,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$J$4:$J$22</c:f>
+              <c:f>'dloads (2)'!$J$5:$J$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3637,7 +3760,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$K$4:$K$22</c:f>
+              <c:f>'dloads (2)'!$K$5:$K$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3691,7 +3814,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$N$4:$N$22</c:f>
+              <c:f>'dloads (2)'!$N$5:$N$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3700,7 +3823,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$O$4:$O$22</c:f>
+              <c:f>'dloads (2)'!$O$5:$O$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3754,7 +3877,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$R$4:$R$22</c:f>
+              <c:f>'dloads (2)'!$R$5:$R$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3763,7 +3886,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$S$4:$S$22</c:f>
+              <c:f>'dloads (2)'!$S$5:$S$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3817,7 +3940,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$V$4:$V$22</c:f>
+              <c:f>'dloads (2)'!$V$5:$V$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3826,7 +3949,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$W$4:$W$22</c:f>
+              <c:f>'dloads (2)'!$W$5:$W$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -6241,7 +6364,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$A$8:$A$27</c:f>
+              <c:f>polygon!$A$10:$A$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6250,7 +6373,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$B$8:$B$27</c:f>
+              <c:f>polygon!$B$10:$B$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6310,7 +6433,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$D$8:$D$27</c:f>
+              <c:f>polygon!$D$10:$D$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6319,7 +6442,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$E$8:$E$27</c:f>
+              <c:f>polygon!$E$10:$E$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6379,7 +6502,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$G$8:$G$27</c:f>
+              <c:f>polygon!$G$10:$G$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6388,7 +6511,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$H$8:$H$27</c:f>
+              <c:f>polygon!$H$10:$H$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6448,7 +6571,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$J$8:$J$27</c:f>
+              <c:f>polygon!$J$10:$J$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6457,7 +6580,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$K$8:$K$27</c:f>
+              <c:f>polygon!$K$10:$K$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6520,7 +6643,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$M$8:$M$27</c:f>
+              <c:f>polygon!$M$10:$M$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6529,7 +6652,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$N$8:$N$27</c:f>
+              <c:f>polygon!$N$10:$N$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6592,7 +6715,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$P$8:$P$27</c:f>
+              <c:f>polygon!$P$10:$P$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6601,7 +6724,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$Q$8:$Q$27</c:f>
+              <c:f>polygon!$Q$10:$Q$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6664,7 +6787,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$S$8:$S$27</c:f>
+              <c:f>polygon!$S$10:$S$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6673,7 +6796,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$T$8:$T$27</c:f>
+              <c:f>polygon!$T$10:$T$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6736,7 +6859,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$V$8:$V$27</c:f>
+              <c:f>polygon!$V$10:$V$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6745,7 +6868,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$W$8:$W$27</c:f>
+              <c:f>polygon!$W$10:$W$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6808,7 +6931,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$Y$8:$Y$27</c:f>
+              <c:f>polygon!$Y$10:$Y$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6817,7 +6940,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$Z$8:$Z$27</c:f>
+              <c:f>polygon!$Z$10:$Z$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6880,7 +7003,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AB$8:$AB$27</c:f>
+              <c:f>polygon!$AB$10:$AB$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6889,7 +7012,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AC$8:$AC$27</c:f>
+              <c:f>polygon!$AC$10:$AC$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6949,7 +7072,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AE$8:$AE$27</c:f>
+              <c:f>polygon!$AE$10:$AE$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6958,7 +7081,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AF$8:$AF$27</c:f>
+              <c:f>polygon!$AF$10:$AF$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7018,7 +7141,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AH$8:$AH$27</c:f>
+              <c:f>polygon!$AH$10:$AH$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7027,7 +7150,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AI$8:$AI$27</c:f>
+              <c:f>polygon!$AI$10:$AI$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7087,7 +7210,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AK$8:$AK$27</c:f>
+              <c:f>polygon!$AK$10:$AK$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7096,7 +7219,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AL$8:$AL$27</c:f>
+              <c:f>polygon!$AL$10:$AL$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7156,7 +7279,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AN$8:$AN$27</c:f>
+              <c:f>polygon!$AN$10:$AN$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7165,7 +7288,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AO$8:$AO$27</c:f>
+              <c:f>polygon!$AO$10:$AO$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7225,7 +7348,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AQ$8:$AQ$27</c:f>
+              <c:f>polygon!$AQ$10:$AQ$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7234,7 +7357,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AR$8:$AR$27</c:f>
+              <c:f>polygon!$AR$10:$AR$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -8965,7 +9088,7 @@
         <v>13</v>
       </c>
       <c r="D5" s="30">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -9164,6 +9287,10 @@
       <c r="D21"/>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="C22" s="14" t="s">
+        <v>307</v>
+      </c>
+      <c r="D22" s="1"/>
       <c r="F22" s="1" t="s">
         <v>62</v>
       </c>
@@ -9311,20 +9438,23 @@
   <mergeCells count="1">
     <mergeCell ref="B7:D7"/>
   </mergeCells>
-  <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D22" xr:uid="{4E2B12C7-FE67-3B4F-885D-33F99F4A0D82}">
+      <formula1>"rollers,fixed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{0D3EDF25-93C5-C944-8126-8CC9B17A21FC}">
       <formula1>$D$50:$D$51</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9" xr:uid="{4694A1A0-8B80-B646-8FBE-EF2E498B980D}">
       <formula1>$D$54:$D$57</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D17" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D17" xr:uid="{0356D3C6-ECF7-2D4C-8DB0-E3BFC9D663DB}">
       <formula1>$D$60:$D$61</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D14" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D14" xr:uid="{BDB1B4FF-9C3D-5F43-BB1B-429406E4C3E1}">
       <formula1>$D$64:$D$71</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D18" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D18" xr:uid="{8A75E61B-C3DC-0F4A-869A-1DA1855E5B34}">
       <formula1>$D$74:$D$78</formula1>
     </dataValidation>
   </dataValidations>
@@ -9334,7 +9464,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="B2:X22"/>
+  <dimension ref="B2:X23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -9384,80 +9514,92 @@
       <c r="X2" s="62"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="C3" s="58"/>
+      <c r="D3" s="39"/>
+      <c r="F3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="G3" s="58"/>
+      <c r="H3" s="39"/>
+      <c r="J3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="K3" s="58"/>
+      <c r="L3" s="39"/>
+      <c r="N3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="O3" s="58"/>
+      <c r="P3" s="39"/>
+      <c r="R3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="S3" s="58"/>
+      <c r="T3" s="39"/>
+      <c r="V3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="W3" s="58"/>
+      <c r="X3" s="39"/>
+    </row>
+    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="T4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="V3" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="W3" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="X3" s="2" t="s">
+      <c r="X4" s="2" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="3"/>
@@ -9819,15 +9961,46 @@
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
     </row>
+    <row r="23" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="R23" s="3"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
+      <c r="V23" s="3"/>
+      <c r="W23" s="3"/>
+      <c r="X23" s="3"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="12">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="V2:X2"/>
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="N2:P2"/>
     <mergeCell ref="R2:T2"/>
     <mergeCell ref="F2:H2"/>
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="R3:S3"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3 H3 L3 P3 T3 X3" xr:uid="{00000000-0002-0000-0900-000000000000}">
+      <formula1>"normal,vertical"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -14634,84 +14807,84 @@
     <mergeCell ref="AG9:AP9"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:K52 AB11:AF52">
-    <cfRule type="expression" dxfId="19" priority="6">
+    <cfRule type="expression" dxfId="34" priority="6">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="7">
+    <cfRule type="expression" dxfId="33" priority="7">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11:L52 O11:R52">
-    <cfRule type="expression" dxfId="17" priority="19">
+    <cfRule type="expression" dxfId="32" priority="19">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="16" priority="8">
+    <cfRule type="expression" dxfId="31" priority="8">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="15" priority="9">
+    <cfRule type="expression" dxfId="30" priority="9">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="14" priority="10">
+    <cfRule type="expression" dxfId="29" priority="10">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P11:P52">
-    <cfRule type="expression" dxfId="13" priority="13">
+    <cfRule type="expression" dxfId="28" priority="13">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="27" priority="23">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="26" priority="24">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="S11:V52">
-    <cfRule type="expression" dxfId="12" priority="11">
+    <cfRule type="expression" dxfId="25" priority="11">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W11:Z52">
-    <cfRule type="expression" dxfId="11" priority="12">
+    <cfRule type="expression" dxfId="24" priority="12">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB11:AF52">
-    <cfRule type="expression" dxfId="10" priority="21">
+    <cfRule type="expression" dxfId="23" priority="21">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC11:AC52">
-    <cfRule type="expression" dxfId="9" priority="14">
+    <cfRule type="expression" dxfId="22" priority="14">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="8" priority="15">
+    <cfRule type="expression" dxfId="21" priority="15">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE11:AF52">
-    <cfRule type="expression" dxfId="7" priority="16">
+    <cfRule type="expression" dxfId="20" priority="16">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="6" priority="17">
+    <cfRule type="expression" dxfId="19" priority="17">
       <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM11:AN52">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="18" priority="1">
       <formula>$AJ11="lf"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="1" priority="23">
-      <formula>$E11="cp"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="24">
-      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -14731,7 +14904,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A2:AR27"/>
+  <dimension ref="A2:AR28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="10.83203125" style="1" customWidth="1"/>
@@ -14765,6 +14938,9 @@
       <c r="D2" s="24" t="s">
         <v>160</v>
       </c>
+      <c r="N2" s="24" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="inlineStr">
@@ -15024,152 +15200,178 @@
       <c r="AR6" s="57"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="B7" s="37"/>
+      <c r="D7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="E7" s="37"/>
+      <c r="G7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="H7" s="37"/>
+      <c r="J7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="K7" s="37"/>
+      <c r="M7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="N7" s="37"/>
+      <c r="P7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="Q7" s="37"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="T7" s="37"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="W7" s="37"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="Z7" s="37"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AC7" s="37"/>
+      <c r="AE7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AF7" s="37"/>
+      <c r="AG7" s="1"/>
+      <c r="AH7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AI7" s="37"/>
+      <c r="AJ7" s="1"/>
+      <c r="AK7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AL7" s="37"/>
+      <c r="AM7" s="1"/>
+      <c r="AN7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AO7" s="37"/>
+      <c r="AP7" s="1"/>
+      <c r="AQ7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AR7" s="37"/>
+    </row>
+    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="M8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="N8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="P8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="Q8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="R7" s="1"/>
-      <c r="S7" s="2" t="s">
+      <c r="R8" s="1"/>
+      <c r="S8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="T7" s="2" t="s">
+      <c r="T8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="U7" s="1"/>
-      <c r="V7" s="2" t="s">
+      <c r="U8" s="1"/>
+      <c r="V8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="W7" s="2" t="s">
+      <c r="W8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="X7" s="1"/>
-      <c r="Y7" s="2" t="s">
+      <c r="X8" s="1"/>
+      <c r="Y8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="Z7" s="2" t="s">
+      <c r="Z8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AA7" s="1"/>
-      <c r="AB7" s="2" t="s">
+      <c r="AA8" s="1"/>
+      <c r="AB8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AC7" s="2" t="s">
+      <c r="AC8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AE7" s="2" t="s">
+      <c r="AE8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AF7" s="2" t="s">
+      <c r="AF8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AG7" s="1"/>
-      <c r="AH7" s="2" t="s">
+      <c r="AG8" s="1"/>
+      <c r="AH8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AI7" s="2" t="s">
+      <c r="AI8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AJ7" s="1"/>
-      <c r="AK7" s="2" t="s">
+      <c r="AJ8" s="1"/>
+      <c r="AK8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AL7" s="2" t="s">
+      <c r="AL8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AM7" s="1"/>
-      <c r="AN7" s="2" t="s">
+      <c r="AM8" s="1"/>
+      <c r="AN8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AO7" s="2" t="s">
+      <c r="AO8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AP7" s="1"/>
-      <c r="AQ7" s="2" t="s">
+      <c r="AP8" s="1"/>
+      <c r="AQ8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AR7" s="2" t="s">
+      <c r="AR8" s="2" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="B8" s="3">
-        <v>53.0</v>
-      </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="1"/>
-      <c r="S8" s="16"/>
-      <c r="T8" s="17"/>
-      <c r="U8" s="1"/>
-      <c r="V8" s="16"/>
-      <c r="W8" s="17"/>
-      <c r="X8" s="1"/>
-      <c r="Y8" s="16"/>
-      <c r="Z8" s="17"/>
-      <c r="AA8" s="1"/>
-      <c r="AB8" s="16"/>
-      <c r="AC8" s="17"/>
-      <c r="AE8" s="3"/>
-      <c r="AF8" s="3"/>
-      <c r="AG8" s="1"/>
-      <c r="AH8" s="16"/>
-      <c r="AI8" s="17"/>
-      <c r="AJ8" s="1"/>
-      <c r="AK8" s="16"/>
-      <c r="AL8" s="17"/>
-      <c r="AM8" s="1"/>
-      <c r="AN8" s="16"/>
-      <c r="AO8" s="17"/>
-      <c r="AP8" s="1"/>
-      <c r="AQ8" s="16"/>
-      <c r="AR8" s="17"/>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="B9" s="3">
         <v>53.0</v>
@@ -15185,38 +15387,38 @@
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
       <c r="R9" s="1"/>
-      <c r="S9" s="18"/>
-      <c r="T9" s="19"/>
+      <c r="S9" s="16"/>
+      <c r="T9" s="17"/>
       <c r="U9" s="1"/>
-      <c r="V9" s="18"/>
-      <c r="W9" s="19"/>
+      <c r="V9" s="16"/>
+      <c r="W9" s="17"/>
       <c r="X9" s="1"/>
-      <c r="Y9" s="18"/>
-      <c r="Z9" s="19"/>
+      <c r="Y9" s="16"/>
+      <c r="Z9" s="17"/>
       <c r="AA9" s="1"/>
-      <c r="AB9" s="18"/>
-      <c r="AC9" s="19"/>
+      <c r="AB9" s="16"/>
+      <c r="AC9" s="17"/>
       <c r="AE9" s="3"/>
       <c r="AF9" s="3"/>
       <c r="AG9" s="1"/>
-      <c r="AH9" s="18"/>
-      <c r="AI9" s="19"/>
+      <c r="AH9" s="16"/>
+      <c r="AI9" s="17"/>
       <c r="AJ9" s="1"/>
-      <c r="AK9" s="18"/>
-      <c r="AL9" s="19"/>
+      <c r="AK9" s="16"/>
+      <c r="AL9" s="17"/>
       <c r="AM9" s="1"/>
-      <c r="AN9" s="18"/>
-      <c r="AO9" s="19"/>
+      <c r="AN9" s="16"/>
+      <c r="AO9" s="17"/>
       <c r="AP9" s="1"/>
-      <c r="AQ9" s="18"/>
-      <c r="AR9" s="19"/>
+      <c r="AQ9" s="16"/>
+      <c r="AR9" s="17"/>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>105.0</v>
+        <v>4.0</v>
       </c>
       <c r="B10" s="3">
-        <v>3.0</v>
+        <v>53.0</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -15257,7 +15459,7 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>115.0</v>
+        <v>105.0</v>
       </c>
       <c r="B11" s="3">
         <v>3.0</v>
@@ -15276,8 +15478,8 @@
       <c r="S11" s="18"/>
       <c r="T11" s="19"/>
       <c r="U11" s="1"/>
-      <c r="V11" s="16"/>
-      <c r="W11" s="17"/>
+      <c r="V11" s="18"/>
+      <c r="W11" s="19"/>
       <c r="X11" s="1"/>
       <c r="Y11" s="18"/>
       <c r="Z11" s="19"/>
@@ -15300,8 +15502,12 @@
       <c r="AR11" s="19"/>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
+      <c r="A12" s="3">
+        <v>115.0</v>
+      </c>
+      <c r="B12" s="3">
+        <v>3.0</v>
+      </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="G12" s="3"/>
@@ -15313,31 +15519,31 @@
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
       <c r="R12" s="1"/>
-      <c r="S12" s="3"/>
-      <c r="T12" s="3"/>
+      <c r="S12" s="18"/>
+      <c r="T12" s="19"/>
       <c r="U12" s="1"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="3"/>
+      <c r="V12" s="16"/>
+      <c r="W12" s="17"/>
       <c r="X12" s="1"/>
-      <c r="Y12" s="3"/>
-      <c r="Z12" s="3"/>
+      <c r="Y12" s="18"/>
+      <c r="Z12" s="19"/>
       <c r="AA12" s="1"/>
-      <c r="AB12" s="3"/>
-      <c r="AC12" s="3"/>
+      <c r="AB12" s="18"/>
+      <c r="AC12" s="19"/>
       <c r="AE12" s="3"/>
       <c r="AF12" s="3"/>
       <c r="AG12" s="1"/>
-      <c r="AH12" s="3"/>
-      <c r="AI12" s="3"/>
+      <c r="AH12" s="18"/>
+      <c r="AI12" s="19"/>
       <c r="AJ12" s="1"/>
-      <c r="AK12" s="3"/>
-      <c r="AL12" s="3"/>
+      <c r="AK12" s="18"/>
+      <c r="AL12" s="19"/>
       <c r="AM12" s="1"/>
-      <c r="AN12" s="3"/>
-      <c r="AO12" s="3"/>
+      <c r="AN12" s="18"/>
+      <c r="AO12" s="19"/>
       <c r="AP12" s="1"/>
-      <c r="AQ12" s="3"/>
-      <c r="AR12" s="3"/>
+      <c r="AQ12" s="18"/>
+      <c r="AR12" s="19"/>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
@@ -15939,6 +16145,46 @@
       <c r="AQ27" s="3"/>
       <c r="AR27" s="3"/>
     </row>
+    <row r="28" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
+      <c r="U28" s="1"/>
+      <c r="V28" s="3"/>
+      <c r="W28" s="3"/>
+      <c r="X28" s="1"/>
+      <c r="Y28" s="3"/>
+      <c r="Z28" s="3"/>
+      <c r="AA28" s="1"/>
+      <c r="AB28" s="3"/>
+      <c r="AC28" s="3"/>
+      <c r="AE28" s="3"/>
+      <c r="AF28" s="3"/>
+      <c r="AG28" s="1"/>
+      <c r="AH28" s="3"/>
+      <c r="AI28" s="3"/>
+      <c r="AJ28" s="1"/>
+      <c r="AK28" s="3"/>
+      <c r="AL28" s="3"/>
+      <c r="AM28" s="1"/>
+      <c r="AN28" s="3"/>
+      <c r="AO28" s="3"/>
+      <c r="AP28" s="1"/>
+      <c r="AQ28" s="3"/>
+      <c r="AR28" s="3"/>
+    </row>
   </sheetData>
   <mergeCells count="30">
     <mergeCell ref="D4:E4"/>
@@ -15978,7 +16224,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A2:AR27"/>
+  <dimension ref="A2:AR29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="10.83203125" style="1" customWidth="1"/>
@@ -16007,7 +16253,7 @@
         <v>179</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
@@ -16088,411 +16334,477 @@
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="B5" s="39">
-        <v>-3</v>
+        <v>198</v>
+      </c>
+      <c r="B5" s="39" t="inlineStr">
+        <is>
+          <t>ssr elastic</t>
+        </is>
       </c>
       <c r="D5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="E5" s="39">
-        <v>-3</v>
+        <v>198</v>
+      </c>
+      <c r="E5" s="39" t="inlineStr">
+        <is>
+          <t>ssr elastic</t>
+        </is>
       </c>
       <c r="G5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="H5" s="39">
-        <v>-3</v>
+        <v>198</v>
+      </c>
+      <c r="H5" s="39" t="inlineStr">
+        <is>
+          <t>ssr elastic</t>
+        </is>
       </c>
       <c r="J5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="K5" s="39">
-        <v>4</v>
+        <v>198</v>
+      </c>
+      <c r="K5" s="39" t="s">
+        <v>305</v>
       </c>
       <c r="M5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="N5" s="39">
-        <v>5</v>
+        <v>198</v>
+      </c>
+      <c r="N5" s="39" t="s">
+        <v>305</v>
       </c>
       <c r="P5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="Q5" s="39">
-        <v>6</v>
+        <v>198</v>
+      </c>
+      <c r="Q5" s="39" t="s">
+        <v>305</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="T5" s="39">
-        <v>7</v>
+        <v>198</v>
+      </c>
+      <c r="T5" s="39" t="s">
+        <v>305</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="W5" s="39">
-        <v>8</v>
+        <v>198</v>
+      </c>
+      <c r="W5" s="39" t="s">
+        <v>305</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="Z5" s="39">
-        <v>9</v>
+        <v>198</v>
+      </c>
+      <c r="Z5" s="39" t="s">
+        <v>305</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AC5" s="39">
-        <v>10</v>
+        <v>198</v>
+      </c>
+      <c r="AC5" s="39" t="s">
+        <v>305</v>
       </c>
       <c r="AE5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AF5" s="39">
-        <v>11</v>
+        <v>198</v>
+      </c>
+      <c r="AF5" s="39" t="s">
+        <v>305</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AI5" s="39">
-        <v>12</v>
+        <v>198</v>
+      </c>
+      <c r="AI5" s="39" t="s">
+        <v>305</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AL5" s="39">
-        <v>13</v>
+        <v>198</v>
+      </c>
+      <c r="AL5" s="39" t="s">
+        <v>305</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AO5" s="39">
-        <v>14</v>
+        <v>198</v>
+      </c>
+      <c r="AO5" s="39" t="s">
+        <v>305</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="AR5" s="39" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="6" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A6" s="38" t="s">
         <v>176</v>
       </c>
-      <c r="AR5" s="39">
+      <c r="B6" s="39"/>
+      <c r="D6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="E6" s="39"/>
+      <c r="G6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="H6" s="39"/>
+      <c r="J6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="K6" s="39">
+        <v>4</v>
+      </c>
+      <c r="M6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="N6" s="39">
+        <v>5</v>
+      </c>
+      <c r="P6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q6" s="39">
+        <v>6</v>
+      </c>
+      <c r="R6" s="1"/>
+      <c r="S6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="T6" s="39">
+        <v>7</v>
+      </c>
+      <c r="U6" s="1"/>
+      <c r="V6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="W6" s="39">
+        <v>8</v>
+      </c>
+      <c r="X6" s="1"/>
+      <c r="Y6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="Z6" s="39">
+        <v>9</v>
+      </c>
+      <c r="AA6" s="1"/>
+      <c r="AB6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AC6" s="39">
+        <v>10</v>
+      </c>
+      <c r="AE6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AF6" s="39">
+        <v>11</v>
+      </c>
+      <c r="AG6" s="1"/>
+      <c r="AH6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AI6" s="39">
+        <v>12</v>
+      </c>
+      <c r="AJ6" s="1"/>
+      <c r="AK6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AL6" s="39">
+        <v>13</v>
+      </c>
+      <c r="AM6" s="1"/>
+      <c r="AN6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AO6" s="39">
+        <v>14</v>
+      </c>
+      <c r="AP6" s="1"/>
+      <c r="AQ6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AR6" s="39">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="58" t="str">
-        <f>IF(B5=-1,"SSR reduce",IF(B5=-2,"SSR hold",IF(B5=-3,"SSR elastic",_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+    <row r="7" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A7" s="58" t="str">
+        <f>IF(OR(B5="",B5="material"),_xlfn.XLOOKUP(B6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="B6" s="57"/>
-      <c r="D6" s="58" t="str">
-        <f>IF(E5=-1,"SSR reduce",IF(E5=-2,"SSR hold",IF(E5=-3,"SSR elastic",_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="B7" s="57"/>
+      <c r="D7" s="58" t="str">
+        <f>IF(OR(E5="",E5="material"),_xlfn.XLOOKUP(E6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="E6" s="57"/>
-      <c r="G6" s="58" t="str">
-        <f>IF(H5=-1,"SSR reduce",IF(H5=-2,"SSR hold",IF(H5=-3,"SSR elastic",_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="E7" s="57"/>
+      <c r="G7" s="58" t="str">
+        <f>IF(OR(H5="",H5="material"),_xlfn.XLOOKUP(H6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="H6" s="57"/>
-      <c r="J6" s="58" t="str">
-        <f>IF(K5=-1,"SSR reduce",IF(K5=-2,"SSR hold",IF(K5=-3,"SSR elastic",_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="H7" s="57"/>
+      <c r="J7" s="58" t="str">
+        <f>IF(OR(K5="",K5="material"),_xlfn.XLOOKUP(K6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="K6" s="57"/>
-      <c r="M6" s="58" t="str">
-        <f>IF(N5=-1,"SSR reduce",IF(N5=-2,"SSR hold",IF(N5=-3,"SSR elastic",_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="K7" s="57"/>
+      <c r="M7" s="58" t="str">
+        <f>IF(OR(N5="",N5="material"),_xlfn.XLOOKUP(N6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="N6" s="57"/>
-      <c r="P6" s="58" t="str">
-        <f>IF(Q5=-1,"SSR reduce",IF(Q5=-2,"SSR hold",IF(Q5=-3,"SSR elastic",_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="N7" s="57"/>
+      <c r="P7" s="58" t="str">
+        <f>IF(OR(Q5="",Q5="material"),_xlfn.XLOOKUP(Q6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="Q6" s="57"/>
-      <c r="R6" s="1"/>
-      <c r="S6" s="58" t="str">
-        <f>IF(T5=-1,"SSR reduce",IF(T5=-2,"SSR hold",IF(T5=-3,"SSR elastic",_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="Q7" s="57"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="58" t="str">
+        <f>IF(OR(T5="",T5="material"),_xlfn.XLOOKUP(T6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="T6" s="57"/>
-      <c r="U6" s="1"/>
-      <c r="V6" s="58" t="str">
-        <f>IF(W5=-1,"SSR reduce",IF(W5=-2,"SSR hold",IF(W5=-3,"SSR elastic",_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="T7" s="57"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="58" t="str">
+        <f>IF(OR(W5="",W5="material"),_xlfn.XLOOKUP(W6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="W6" s="57"/>
-      <c r="X6" s="1"/>
-      <c r="Y6" s="58" t="str">
-        <f>IF(Z5=-1,"SSR reduce",IF(Z5=-2,"SSR hold",IF(Z5=-3,"SSR elastic",_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="W7" s="57"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="58" t="str">
+        <f>IF(OR(Z5="",Z5="material"),_xlfn.XLOOKUP(Z6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="Z6" s="57"/>
-      <c r="AA6" s="1"/>
-      <c r="AB6" s="58" t="str">
-        <f>IF(AC5=-1,"SSR reduce",IF(AC5=-2,"SSR hold",IF(AC5=-3,"SSR elastic",_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="Z7" s="57"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="58" t="str">
+        <f>IF(OR(AC5="",AC5="material"),_xlfn.XLOOKUP(AC6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="AC6" s="57"/>
-      <c r="AE6" s="58" t="str">
-        <f>IF(AF5=-1,"SSR reduce",IF(AF5=-2,"SSR hold",IF(AF5=-3,"SSR elastic",_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="AC7" s="57"/>
+      <c r="AE7" s="58" t="str">
+        <f>IF(OR(AF5="",AF5="material"),_xlfn.XLOOKUP(AF6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="AF6" s="57"/>
-      <c r="AG6" s="1"/>
-      <c r="AH6" s="58" t="str">
-        <f>IF(AI5=-1,"SSR reduce",IF(AI5=-2,"SSR hold",IF(AI5=-3,"SSR elastic",_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="AF7" s="57"/>
+      <c r="AG7" s="1"/>
+      <c r="AH7" s="58" t="str">
+        <f>IF(OR(AI5="",AI5="material"),_xlfn.XLOOKUP(AI6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="AI6" s="57"/>
-      <c r="AJ6" s="1"/>
-      <c r="AK6" s="58" t="str">
-        <f>IF(AL5=-1,"SSR reduce",IF(AL5=-2,"SSR hold",IF(AL5=-3,"SSR elastic",_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="AI7" s="57"/>
+      <c r="AJ7" s="1"/>
+      <c r="AK7" s="58" t="str">
+        <f>IF(OR(AL5="",AL5="material"),_xlfn.XLOOKUP(AL6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="AL6" s="57"/>
-      <c r="AM6" s="1"/>
-      <c r="AN6" s="58" t="str">
-        <f>IF(AO5=-1,"SSR reduce",IF(AO5=-2,"SSR hold",IF(AO5=-3,"SSR elastic",_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="AL7" s="57"/>
+      <c r="AM7" s="1"/>
+      <c r="AN7" s="58" t="str">
+        <f>IF(OR(AO5="",AO5="material"),_xlfn.XLOOKUP(AO6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="AO6" s="57"/>
-      <c r="AP6" s="1"/>
-      <c r="AQ6" s="58" t="str">
-        <f>IF(AR5=-1,"SSR reduce",IF(AR5=-2,"SSR hold",IF(AR5=-3,"SSR elastic",_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="AO7" s="57"/>
+      <c r="AP7" s="1"/>
+      <c r="AQ7" s="58" t="str">
+        <f>IF(OR(AR5="",AR5="material"),_xlfn.XLOOKUP(AR6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
         <v/>
       </c>
-      <c r="AR6" s="57"/>
-    </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+      <c r="AR7" s="57"/>
+    </row>
+    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="B8" s="39"/>
+      <c r="D8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="E8" s="39"/>
+      <c r="G8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="H8" s="39"/>
+      <c r="J8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="K8" s="39"/>
+      <c r="M8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="N8" s="39"/>
+      <c r="P8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="Q8" s="39"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="T8" s="39"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="W8" s="39"/>
+      <c r="X8" s="1"/>
+      <c r="Y8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="Z8" s="39"/>
+      <c r="AA8" s="1"/>
+      <c r="AB8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AC8" s="39"/>
+      <c r="AE8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AF8" s="39"/>
+      <c r="AG8" s="1"/>
+      <c r="AH8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AI8" s="39"/>
+      <c r="AJ8" s="1"/>
+      <c r="AK8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AL8" s="39"/>
+      <c r="AM8" s="1"/>
+      <c r="AN8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AO8" s="39"/>
+      <c r="AP8" s="1"/>
+      <c r="AQ8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AR8" s="39"/>
+    </row>
+    <row r="9" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="K9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="M9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="N9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="P9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="Q9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="R7" s="1"/>
-      <c r="S7" s="2" t="s">
+      <c r="R9" s="1"/>
+      <c r="S9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="T7" s="2" t="s">
+      <c r="T9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="U7" s="1"/>
-      <c r="V7" s="2" t="s">
+      <c r="U9" s="1"/>
+      <c r="V9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="W7" s="2" t="s">
+      <c r="W9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="X7" s="1"/>
-      <c r="Y7" s="2" t="s">
+      <c r="X9" s="1"/>
+      <c r="Y9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="Z7" s="2" t="s">
+      <c r="Z9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AA7" s="1"/>
-      <c r="AB7" s="2" t="s">
+      <c r="AA9" s="1"/>
+      <c r="AB9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AC7" s="2" t="s">
+      <c r="AC9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AE7" s="2" t="s">
+      <c r="AE9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AF7" s="2" t="s">
+      <c r="AF9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AG7" s="1"/>
-      <c r="AH7" s="2" t="s">
+      <c r="AG9" s="1"/>
+      <c r="AH9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AI7" s="2" t="s">
+      <c r="AI9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AJ7" s="1"/>
-      <c r="AK7" s="2" t="s">
+      <c r="AJ9" s="1"/>
+      <c r="AK9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AL7" s="2" t="s">
+      <c r="AL9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AM7" s="1"/>
-      <c r="AN7" s="2" t="s">
+      <c r="AM9" s="1"/>
+      <c r="AN9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AO7" s="2" t="s">
+      <c r="AO9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AP7" s="1"/>
-      <c r="AQ7" s="2" t="s">
+      <c r="AP9" s="1"/>
+      <c r="AQ9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AR7" s="2" t="s">
+      <c r="AR9" s="2" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="B8" s="3">
-        <v>53.0</v>
-      </c>
-      <c r="D8" s="3">
-        <v>105.0</v>
-      </c>
-      <c r="E8" s="3">
-        <v>2.8</v>
-      </c>
-      <c r="G8" s="3">
-        <v>20.0</v>
-      </c>
-      <c r="H8" s="3">
-        <v>16.0</v>
-      </c>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="1"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
-      <c r="U8" s="1"/>
-      <c r="V8" s="3"/>
-      <c r="W8" s="3"/>
-      <c r="X8" s="1"/>
-      <c r="Y8" s="3"/>
-      <c r="Z8" s="3"/>
-      <c r="AA8" s="1"/>
-      <c r="AB8" s="3"/>
-      <c r="AC8" s="3"/>
-      <c r="AE8" s="3"/>
-      <c r="AF8" s="3"/>
-      <c r="AG8" s="1"/>
-      <c r="AH8" s="3"/>
-      <c r="AI8" s="3"/>
-      <c r="AJ8" s="1"/>
-      <c r="AK8" s="3"/>
-      <c r="AL8" s="3"/>
-      <c r="AM8" s="1"/>
-      <c r="AN8" s="3"/>
-      <c r="AO8" s="3"/>
-      <c r="AP8" s="1"/>
-      <c r="AQ8" s="3"/>
-      <c r="AR8" s="3"/>
-    </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="B9" s="3">
-        <v>-10.0</v>
-      </c>
-      <c r="D9" s="3">
-        <v>105.0</v>
-      </c>
-      <c r="E9" s="3">
-        <v>-10.0</v>
-      </c>
-      <c r="G9" s="3">
-        <v>40.0</v>
-      </c>
-      <c r="H9" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="1"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
-      <c r="U9" s="1"/>
-      <c r="V9" s="3"/>
-      <c r="W9" s="3"/>
-      <c r="X9" s="1"/>
-      <c r="Y9" s="3"/>
-      <c r="Z9" s="3"/>
-      <c r="AA9" s="1"/>
-      <c r="AB9" s="3"/>
-      <c r="AC9" s="3"/>
-      <c r="AE9" s="3"/>
-      <c r="AF9" s="3"/>
-      <c r="AG9" s="1"/>
-      <c r="AH9" s="3"/>
-      <c r="AI9" s="3"/>
-      <c r="AJ9" s="1"/>
-      <c r="AK9" s="3"/>
-      <c r="AL9" s="3"/>
-      <c r="AM9" s="1"/>
-      <c r="AN9" s="3"/>
-      <c r="AO9" s="3"/>
-      <c r="AP9" s="1"/>
-      <c r="AQ9" s="3"/>
-      <c r="AR9" s="3"/>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="B10" s="3">
-        <v>-9.8681</v>
+        <v>53.0</v>
       </c>
       <c r="D10" s="3">
-        <v>115.0</v>
+        <v>105.0</v>
       </c>
       <c r="E10" s="3">
-        <v>-10.0</v>
+        <v>2.8</v>
       </c>
       <c r="G10" s="3">
-        <v>60.0</v>
+        <v>20.0</v>
       </c>
       <c r="H10" s="3">
-        <v>4.0</v>
+        <v>16.0</v>
       </c>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
@@ -16529,22 +16841,22 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="B11" s="3">
-        <v>53.0</v>
+        <v>-10.0</v>
       </c>
       <c r="D11" s="3">
-        <v>115.0</v>
+        <v>105.0</v>
       </c>
       <c r="E11" s="3">
-        <v>2.8</v>
+        <v>-10.0</v>
       </c>
       <c r="G11" s="3">
-        <v>80.0</v>
+        <v>40.0</v>
       </c>
       <c r="H11" s="3">
-        <v>1.0</v>
+        <v>8.0</v>
       </c>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
@@ -16580,15 +16892,23 @@
       <c r="AR11" s="3"/>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
+      <c r="A12" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="B12" s="3">
+        <v>-9.8681</v>
+      </c>
+      <c r="D12" s="3">
+        <v>115.0</v>
+      </c>
+      <c r="E12" s="3">
+        <v>-10.0</v>
+      </c>
       <c r="G12" s="3">
-        <v>102.392</v>
+        <v>60.0</v>
       </c>
       <c r="H12" s="3">
-        <v>4.09622</v>
+        <v>4.0</v>
       </c>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
@@ -16624,15 +16944,23 @@
       <c r="AR12" s="3"/>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
+      <c r="A13" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="B13" s="3">
+        <v>53.0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>115.0</v>
+      </c>
+      <c r="E13" s="3">
+        <v>2.8</v>
+      </c>
       <c r="G13" s="3">
-        <v>6.53543</v>
+        <v>80.0</v>
       </c>
       <c r="H13" s="3">
-        <v>51.7398</v>
+        <v>1.0</v>
       </c>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
@@ -16672,8 +17000,12 @@
       <c r="B14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
+      <c r="G14" s="3">
+        <v>102.392</v>
+      </c>
+      <c r="H14" s="3">
+        <v>4.09622</v>
+      </c>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
       <c r="M14" s="3"/>
@@ -16712,8 +17044,12 @@
       <c r="B15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
+      <c r="G15" s="3">
+        <v>6.53543</v>
+      </c>
+      <c r="H15" s="3">
+        <v>51.7398</v>
+      </c>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
       <c r="M15" s="3"/>
@@ -17227,39 +17563,199 @@
       <c r="AQ27" s="3"/>
       <c r="AR27" s="3"/>
     </row>
+    <row r="28" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
+      <c r="U28" s="1"/>
+      <c r="V28" s="3"/>
+      <c r="W28" s="3"/>
+      <c r="X28" s="1"/>
+      <c r="Y28" s="3"/>
+      <c r="Z28" s="3"/>
+      <c r="AA28" s="1"/>
+      <c r="AB28" s="3"/>
+      <c r="AC28" s="3"/>
+      <c r="AE28" s="3"/>
+      <c r="AF28" s="3"/>
+      <c r="AG28" s="1"/>
+      <c r="AH28" s="3"/>
+      <c r="AI28" s="3"/>
+      <c r="AJ28" s="1"/>
+      <c r="AK28" s="3"/>
+      <c r="AL28" s="3"/>
+      <c r="AM28" s="1"/>
+      <c r="AN28" s="3"/>
+      <c r="AO28" s="3"/>
+      <c r="AP28" s="1"/>
+      <c r="AQ28" s="3"/>
+      <c r="AR28" s="3"/>
+    </row>
+    <row r="29" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A29" s="3"/>
+      <c r="B29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3"/>
+      <c r="R29" s="1"/>
+      <c r="S29" s="3"/>
+      <c r="T29" s="3"/>
+      <c r="U29" s="1"/>
+      <c r="V29" s="3"/>
+      <c r="W29" s="3"/>
+      <c r="X29" s="1"/>
+      <c r="Y29" s="3"/>
+      <c r="Z29" s="3"/>
+      <c r="AA29" s="1"/>
+      <c r="AB29" s="3"/>
+      <c r="AC29" s="3"/>
+      <c r="AE29" s="3"/>
+      <c r="AF29" s="3"/>
+      <c r="AG29" s="1"/>
+      <c r="AH29" s="3"/>
+      <c r="AI29" s="3"/>
+      <c r="AJ29" s="1"/>
+      <c r="AK29" s="3"/>
+      <c r="AL29" s="3"/>
+      <c r="AM29" s="1"/>
+      <c r="AN29" s="3"/>
+      <c r="AO29" s="3"/>
+      <c r="AP29" s="1"/>
+      <c r="AQ29" s="3"/>
+      <c r="AR29" s="3"/>
+    </row>
   </sheetData>
   <mergeCells count="30">
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="P4:Q4"/>
     <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="AN7:AO7"/>
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
     <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="V7:W7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="AH7:AI7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="Y7:Z7"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="AK7:AL7"/>
+    <mergeCell ref="AE7:AF7"/>
+    <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
     <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="P7:Q7"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6 A7:B7">
+    <cfRule type="expression" dxfId="17" priority="1">
+      <formula>AND($B$5&lt;&gt;"",$B$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6 D7:E7">
+    <cfRule type="expression" dxfId="16" priority="2">
+      <formula>AND($E$5&lt;&gt;"",$E$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H6 G7:H7">
+    <cfRule type="expression" dxfId="15" priority="3">
+      <formula>AND($H$5&lt;&gt;"",$H$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K6 J7:K7">
+    <cfRule type="expression" dxfId="14" priority="4">
+      <formula>AND($K$5&lt;&gt;"",$K$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N6 M7:N7">
+    <cfRule type="expression" dxfId="13" priority="5">
+      <formula>AND($N$5&lt;&gt;"",$N$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q6 P7:Q7">
+    <cfRule type="expression" dxfId="12" priority="6">
+      <formula>AND($Q$5&lt;&gt;"",$Q$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T6 S7:T7">
+    <cfRule type="expression" dxfId="11" priority="7">
+      <formula>AND($T$5&lt;&gt;"",$T$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W6 V7:W7">
+    <cfRule type="expression" dxfId="10" priority="8">
+      <formula>AND($W$5&lt;&gt;"",$W$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z6 Y7:Z7">
+    <cfRule type="expression" dxfId="9" priority="9">
+      <formula>AND($Z$5&lt;&gt;"",$Z$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC6 AB7:AC7">
+    <cfRule type="expression" dxfId="8" priority="10">
+      <formula>AND($AC$5&lt;&gt;"",$AC$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AF6 AE7:AF7">
+    <cfRule type="expression" dxfId="7" priority="11">
+      <formula>AND($AF$5&lt;&gt;"",$AF$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI6 AH7:AI7">
+    <cfRule type="expression" dxfId="6" priority="12">
+      <formula>AND($AI$5&lt;&gt;"",$AI$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL6 AK7:AL7">
+    <cfRule type="expression" dxfId="5" priority="13">
+      <formula>AND($AL$5&lt;&gt;"",$AL$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO6 AN7:AO7">
+    <cfRule type="expression" dxfId="4" priority="14">
+      <formula>AND($AO$5&lt;&gt;"",$AO$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AR6 AQ7:AR7">
+    <cfRule type="expression" dxfId="3" priority="15">
+      <formula>AND($AR$5&lt;&gt;"",$AR$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5 E5 H5 K5 N5 Q5 T5 W5 Z5 AC5 AF5 AI5 AL5 AO5 AR5" xr:uid="{00000000-0002-0000-0400-000000000000}">
+      <formula1>"material,ssr reduce,ssr hold,ssr elastic,refine"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -17707,17 +18203,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E42">
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17940,7 +18436,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="B2:X22"/>
+  <dimension ref="B2:X23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -17990,80 +18486,92 @@
       <c r="X2" s="62"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="C3" s="58"/>
+      <c r="D3" s="39"/>
+      <c r="F3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="G3" s="58"/>
+      <c r="H3" s="39"/>
+      <c r="J3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="K3" s="58"/>
+      <c r="L3" s="39"/>
+      <c r="N3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="O3" s="58"/>
+      <c r="P3" s="39"/>
+      <c r="R3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="S3" s="58"/>
+      <c r="T3" s="39"/>
+      <c r="V3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="W3" s="58"/>
+      <c r="X3" s="39"/>
+    </row>
+    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="T4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="V3" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="W3" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="X3" s="2" t="s">
+      <c r="X4" s="2" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="3"/>
@@ -18425,15 +18933,46 @@
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
     </row>
+    <row r="23" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="R23" s="3"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
+      <c r="V23" s="3"/>
+      <c r="W23" s="3"/>
+      <c r="X23" s="3"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="12">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="V2:X2"/>
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="N2:P2"/>
     <mergeCell ref="R2:T2"/>
     <mergeCell ref="F2:H2"/>
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="R3:S3"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3 H3 L3 P3 T3 X3" xr:uid="{00000000-0002-0000-0800-000000000000}">
+      <formula1>"normal,vertical"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>